<commit_message>
Included measurements for Phase 2, added in different excel sheets
</commit_message>
<xml_diff>
--- a/Measurements/Measurements_Sensitec.xlsx
+++ b/Measurements/Measurements_Sensitec.xlsx
@@ -5,16 +5,18 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\IlhanK\Desktop\FP\uz_per_external_current_sensing\Measurements\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\IlhanK\Documents\uz_per_external_current_sensing\Measurements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65A9B8E2-F72D-45F9-9A11-5151F68DE96A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A12698E6-35D3-4F5B-A943-2AA8FFABB817}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="71895" yWindow="-12150" windowWidth="14610" windowHeight="15420" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57480" yWindow="-12270" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="phase1_with_R5_R2" sheetId="1" r:id="rId1"/>
+    <sheet name="phase1_with_0Ohm" sheetId="2" r:id="rId2"/>
+    <sheet name="phase2_with_R5_R2" sheetId="3" r:id="rId3"/>
+    <sheet name="phase2_with_0Ohm" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="34">
   <si>
     <t>I_IN (A)</t>
   </si>
@@ -122,6 +124,24 @@
   <si>
     <t>Gain*VIN</t>
   </si>
+  <si>
+    <t>Pin 2 ( V_OCM)</t>
+  </si>
+  <si>
+    <t>I_OUT_P</t>
+  </si>
+  <si>
+    <t>I_OUT_N</t>
+  </si>
+  <si>
+    <t>PHASE2</t>
+  </si>
+  <si>
+    <t>Deviation (%)</t>
+  </si>
+  <si>
+    <t>R2 and R5 stayed as is in schematic</t>
+  </si>
 </sst>
 </file>
 
@@ -130,7 +150,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -171,6 +191,27 @@
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="20"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -237,7 +278,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -273,13 +314,32 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -414,7 +474,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$C$6:$C$26</c:f>
+              <c:f>phase1_with_R5_R2!$C$6:$C$26</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="21"/>
@@ -486,7 +546,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$M$6:$M$26</c:f>
+              <c:f>phase1_with_R5_R2!$M$6:$M$26</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="21"/>
@@ -595,7 +655,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$C$6:$C$26</c:f>
+              <c:f>phase1_with_R5_R2!$C$6:$C$26</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="21"/>
@@ -667,7 +727,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$N$6:$N$26</c:f>
+              <c:f>phase1_with_R5_R2!$N$6:$N$26</c:f>
               <c:numCache>
                 <c:formatCode>0.0000</c:formatCode>
                 <c:ptCount val="21"/>
@@ -1192,7 +1252,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet2!$B$6:$B$32</c:f>
+              <c:f>phase1_with_0Ohm!$B$6:$B$32</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="27"/>
@@ -1282,7 +1342,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet2!$J$6:$J$32</c:f>
+              <c:f>phase1_with_0Ohm!$J$6:$J$32</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="27"/>
@@ -1293,10 +1353,10 @@
                   <c:v>29.177777777777781</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>20.289999999999996</c:v>
+                  <c:v>20.255000000000003</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>8.862857142857143</c:v>
+                  <c:v>8.8742857142857137</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0.18666666666666093</c:v>
@@ -1350,7 +1410,7 @@
                   <c:v>1.0700000000000043</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>0.94400000000000261</c:v>
+                  <c:v>1.039999999999992</c:v>
                 </c:pt>
                 <c:pt idx="22">
                   <c:v>0.78000000000000291</c:v>
@@ -1692,6 +1752,615 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:sysClr>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>Deviation (%) vs Input Current (A)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="de-DE"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>phase2_with_0Ohm!$C$8:$C$34</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="27"/>
+                <c:pt idx="0">
+                  <c:v>-50</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-45</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-40</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-35</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-30</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-25</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-20</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-15</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-10</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>-8</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>-6</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>-4</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>-2</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>35</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>50</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>phase2_with_0Ohm!$G$8:$G$34</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="27"/>
+                <c:pt idx="0">
+                  <c:v>-4.0000000000084412E-3</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3.1111111111117553E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6.0000000000004494E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.13142857142856965</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.24000000000000318</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.39999999999999153</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.49000000000000155</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.46666666666665968</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.3000000000000012</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1.2000000000000066</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>2.3333333333333357</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>2.5000000000000022</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>4.2000000000000091</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>4.7999999999999989</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>4.0000000000000036</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>3.3333333333333366</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>2.0000000000000018</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>1.419999999999999</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.58666666666666134</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0.60000000000000053</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>0.48000000000000037</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0.2999999999999966</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>0.25714285714285418</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>0.18500000000000183</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>0.16000000000000211</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>0.13199999999999434</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-580D-4C46-8DFD-61C41EDAED4C}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1139084831"/>
+        <c:axId val="1139086751"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1139084831"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="50"/>
+          <c:min val="-50"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="de-DE" sz="1600" b="1"/>
+                  <a:t>Input</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="de-DE" sz="1600" b="1" baseline="0"/>
+                  <a:t> Current (A)</a:t>
+                </a:r>
+                <a:endParaRPr lang="de-DE" sz="1600" b="1"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout>
+            <c:manualLayout>
+              <c:xMode val="edge"/>
+              <c:yMode val="edge"/>
+              <c:x val="0.41617705820441259"/>
+              <c:y val="0.89109111127901952"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="de-DE"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="de-DE"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1139086751"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+        <c:majorUnit val="5"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1139086751"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="de-DE" sz="1600" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:sysClr val="windowText" lastClr="000000">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:sysClr>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t>Error (%)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="de-DE"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="de-DE"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1139084831"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="de-DE"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -1772,6 +2441,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
@@ -2289,6 +2998,522 @@
 </file>
 
 <file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -3373,7 +4598,7 @@
       <xdr:col>31</xdr:col>
       <xdr:colOff>417985</xdr:colOff>
       <xdr:row>56</xdr:row>
-      <xdr:rowOff>66061</xdr:rowOff>
+      <xdr:rowOff>69237</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3415,9 +4640,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>523595</xdr:colOff>
+      <xdr:colOff>526770</xdr:colOff>
       <xdr:row>59</xdr:row>
-      <xdr:rowOff>75033</xdr:rowOff>
+      <xdr:rowOff>75034</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3457,16 +4682,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>191267</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>247295</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>25587</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>24</xdr:col>
-      <xdr:colOff>104919</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>90456</xdr:rowOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>635855</xdr:colOff>
+      <xdr:row>55</xdr:row>
+      <xdr:rowOff>47998</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3489,8 +4714,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9081267" y="3516153"/>
-          <a:ext cx="7870278" cy="3208728"/>
+          <a:off x="852413" y="6356911"/>
+          <a:ext cx="8964235" cy="3605118"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3501,16 +4726,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>464161</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>45674</xdr:rowOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>400101</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>149702</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>24</xdr:col>
-      <xdr:colOff>390180</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>114759</xdr:rowOff>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>326120</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>36318</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -3530,6 +4755,47 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>58943</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>44726</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>496957</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>149087</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{66B52199-998E-6ABF-C061-3F27795C8A0D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3801,7 +5067,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="C2:R27"/>
+  <dimension ref="B1:R27"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.1796875" customWidth="1"/>
@@ -3824,18 +5090,23 @@
     <col min="18" max="18" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="3:17" x14ac:dyDescent="0.35">
+    <row r="1" spans="2:17" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="B1" s="12" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="2:17" x14ac:dyDescent="0.35">
       <c r="Q2" s="9" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="3:17" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:17" x14ac:dyDescent="0.35">
       <c r="Q3" s="10">
         <f>2000/1051</f>
         <v>1.9029495718363463</v>
       </c>
     </row>
-    <row r="4" spans="3:17" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:17" x14ac:dyDescent="0.35">
       <c r="D4" s="8" t="s">
         <v>4</v>
       </c>
@@ -3858,7 +5129,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="3:17" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:17" x14ac:dyDescent="0.35">
       <c r="C5" s="4" t="s">
         <v>0</v>
       </c>
@@ -3900,7 +5171,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="3:17" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:17" x14ac:dyDescent="0.35">
       <c r="C6" s="3">
         <v>-10</v>
       </c>
@@ -3951,7 +5222,7 @@
         <v>-0.24009999999999998</v>
       </c>
     </row>
-    <row r="7" spans="3:17" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:17" x14ac:dyDescent="0.35">
       <c r="C7" s="3">
         <v>-9</v>
       </c>
@@ -4002,7 +5273,7 @@
         <v>-0.21620000000000017</v>
       </c>
     </row>
-    <row r="8" spans="3:17" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:17" x14ac:dyDescent="0.35">
       <c r="C8" s="3">
         <v>-8</v>
       </c>
@@ -4053,7 +5324,7 @@
         <v>-0.19240000000000013</v>
       </c>
     </row>
-    <row r="9" spans="3:17" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:17" x14ac:dyDescent="0.35">
       <c r="C9" s="3">
         <v>-7</v>
       </c>
@@ -4104,7 +5375,7 @@
         <v>-0.16870000000000029</v>
       </c>
     </row>
-    <row r="10" spans="3:17" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:17" x14ac:dyDescent="0.35">
       <c r="C10" s="3">
         <v>-6</v>
       </c>
@@ -4155,7 +5426,7 @@
         <v>-0.14480000000000004</v>
       </c>
     </row>
-    <row r="11" spans="3:17" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:17" x14ac:dyDescent="0.35">
       <c r="C11" s="3">
         <v>-5</v>
       </c>
@@ -4206,7 +5477,7 @@
         <v>-0.12109999999999976</v>
       </c>
     </row>
-    <row r="12" spans="3:17" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:17" x14ac:dyDescent="0.35">
       <c r="C12" s="3">
         <v>-4</v>
       </c>
@@ -4257,7 +5528,7 @@
         <v>-9.7199999999999953E-2</v>
       </c>
     </row>
-    <row r="13" spans="3:17" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:17" x14ac:dyDescent="0.35">
       <c r="C13" s="3">
         <v>-3</v>
       </c>
@@ -4308,7 +5579,7 @@
         <v>-7.3400000000000354E-2</v>
       </c>
     </row>
-    <row r="14" spans="3:17" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:17" x14ac:dyDescent="0.35">
       <c r="C14" s="3">
         <v>-2</v>
       </c>
@@ -4359,7 +5630,7 @@
         <v>-4.9700000000000077E-2</v>
       </c>
     </row>
-    <row r="15" spans="3:17" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:17" x14ac:dyDescent="0.35">
       <c r="C15" s="3">
         <v>-1</v>
       </c>
@@ -4410,7 +5681,7 @@
         <v>-2.5800000000000267E-2</v>
       </c>
     </row>
-    <row r="16" spans="3:17" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:17" x14ac:dyDescent="0.35">
       <c r="C16" s="3">
         <v>0</v>
       </c>
@@ -4991,7 +6262,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4238C765-75F2-4EFE-AC8B-2868F72A3DB3}">
-  <dimension ref="B1:J32"/>
+  <dimension ref="B1:M34"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="7.08984375" bestFit="1" customWidth="1"/>
@@ -5002,941 +6273,2148 @@
     <col min="8" max="8" width="13.36328125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="17.1796875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:10" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="2:13" ht="18.5" x14ac:dyDescent="0.45">
       <c r="B1" s="12" t="s">
         <v>26</v>
       </c>
       <c r="C1" s="12"/>
     </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="C4" s="8" t="s">
+    <row r="4" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="C4" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="15" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B5" s="4" t="s">
+    <row r="5" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B5" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="H5" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="4" t="s">
+      <c r="I5" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="J5" s="4" t="s">
+      <c r="J5" s="17" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="6" spans="2:10" s="15" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="13">
+      <c r="K5" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="L5" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="M5" s="17" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="2:13" s="13" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B6" s="19">
         <v>-50</v>
       </c>
-      <c r="C6" s="14">
+      <c r="C6" s="20">
         <v>1.2462</v>
       </c>
-      <c r="D6" s="14">
+      <c r="D6" s="20">
         <v>2.4950999999999999</v>
       </c>
-      <c r="E6" s="14">
+      <c r="E6" s="20">
         <f>C6-D6</f>
         <v>-1.2488999999999999</v>
       </c>
-      <c r="F6" s="14">
+      <c r="F6" s="20">
         <f>2*E6</f>
         <v>-2.4977999999999998</v>
       </c>
-      <c r="G6" s="13">
+      <c r="G6" s="19">
         <v>-2.5</v>
       </c>
-      <c r="H6" s="14">
+      <c r="H6" s="20">
         <v>-1.5911999999999999</v>
       </c>
-      <c r="I6" s="14">
+      <c r="I6" s="20">
         <f>G6-H6</f>
         <v>-0.90880000000000005</v>
       </c>
-      <c r="J6" s="13">
+      <c r="J6" s="19">
         <f t="shared" ref="J6:J13" si="0">(I6/G6)*100</f>
         <v>36.352000000000004</v>
       </c>
-    </row>
-    <row r="7" spans="2:10" s="15" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="13">
+      <c r="K6" s="19">
+        <v>2.0084</v>
+      </c>
+      <c r="L6" s="21">
+        <v>4.09</v>
+      </c>
+      <c r="M6" s="21">
+        <v>2.4948999999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="2:13" s="13" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B7" s="19">
         <v>-45</v>
       </c>
-      <c r="C7" s="14">
+      <c r="C7" s="20">
         <v>1.3712</v>
       </c>
-      <c r="D7" s="14">
+      <c r="D7" s="20">
         <v>2.4950000000000001</v>
       </c>
-      <c r="E7" s="14">
+      <c r="E7" s="20">
         <f t="shared" ref="E7:E32" si="1">C7-D7</f>
         <v>-1.1238000000000001</v>
       </c>
-      <c r="F7" s="14">
+      <c r="F7" s="20">
         <f t="shared" ref="F7:F32" si="2">2*E7</f>
         <v>-2.2476000000000003</v>
       </c>
-      <c r="G7" s="13">
+      <c r="G7" s="19">
         <v>-2.25</v>
       </c>
-      <c r="H7" s="14">
+      <c r="H7" s="20">
         <v>-1.5934999999999999</v>
       </c>
-      <c r="I7" s="14">
+      <c r="I7" s="20">
         <f t="shared" ref="I7:I13" si="3">G7-H7</f>
         <v>-0.65650000000000008</v>
       </c>
-      <c r="J7" s="13">
+      <c r="J7" s="19">
         <f t="shared" si="0"/>
         <v>29.177777777777781</v>
       </c>
-    </row>
-    <row r="8" spans="2:10" s="15" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="13">
+      <c r="K7" s="19">
+        <v>2.0084</v>
+      </c>
+      <c r="L7" s="21">
+        <v>4.09</v>
+      </c>
+      <c r="M7" s="21">
+        <v>2.4948999999999999</v>
+      </c>
+    </row>
+    <row r="8" spans="2:13" s="13" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B8" s="19">
         <v>-40</v>
       </c>
-      <c r="C8" s="14">
+      <c r="C8" s="20">
         <v>1.4961</v>
       </c>
-      <c r="D8" s="14">
+      <c r="D8" s="20">
         <v>2.4950000000000001</v>
       </c>
-      <c r="E8" s="14">
+      <c r="E8" s="20">
         <f t="shared" si="1"/>
         <v>-0.99890000000000012</v>
       </c>
-      <c r="F8" s="14">
+      <c r="F8" s="20">
         <f t="shared" si="2"/>
         <v>-1.9978000000000002</v>
       </c>
-      <c r="G8" s="13">
+      <c r="G8" s="19">
         <v>-2</v>
       </c>
-      <c r="H8" s="14">
-        <v>-1.5942000000000001</v>
-      </c>
-      <c r="I8" s="14">
+      <c r="H8" s="20">
+        <v>-1.5949</v>
+      </c>
+      <c r="I8" s="20">
         <f t="shared" si="3"/>
-        <v>-0.40579999999999994</v>
-      </c>
-      <c r="J8" s="13">
+        <v>-0.40510000000000002</v>
+      </c>
+      <c r="J8" s="19">
         <f t="shared" si="0"/>
-        <v>20.289999999999996</v>
-      </c>
-    </row>
-    <row r="9" spans="2:10" s="15" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="13">
+        <v>20.255000000000003</v>
+      </c>
+      <c r="K8" s="19">
+        <v>2.0087999999999999</v>
+      </c>
+      <c r="L8" s="21">
+        <v>4.0904999999999996</v>
+      </c>
+      <c r="M8" s="21">
+        <v>2.4948999999999999</v>
+      </c>
+    </row>
+    <row r="9" spans="2:13" s="13" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B9" s="19">
         <v>-35</v>
       </c>
-      <c r="C9" s="14">
+      <c r="C9" s="20">
         <v>1.6212</v>
       </c>
-      <c r="D9" s="14">
+      <c r="D9" s="20">
+        <v>2.4946000000000002</v>
+      </c>
+      <c r="E9" s="20">
+        <f t="shared" si="1"/>
+        <v>-0.87340000000000018</v>
+      </c>
+      <c r="F9" s="20">
+        <f t="shared" si="2"/>
+        <v>-1.7468000000000004</v>
+      </c>
+      <c r="G9" s="19">
+        <v>-1.75</v>
+      </c>
+      <c r="H9" s="20">
+        <v>-1.5947</v>
+      </c>
+      <c r="I9" s="20">
+        <f t="shared" si="3"/>
+        <v>-0.15529999999999999</v>
+      </c>
+      <c r="J9" s="19">
+        <f t="shared" si="0"/>
+        <v>8.8742857142857137</v>
+      </c>
+      <c r="K9" s="19">
+        <v>2.0084</v>
+      </c>
+      <c r="L9" s="21">
+        <v>4.0904999999999996</v>
+      </c>
+      <c r="M9" s="21">
         <v>2.4948999999999999</v>
       </c>
-      <c r="E9" s="14">
+    </row>
+    <row r="10" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B10" s="19">
+        <v>-30</v>
+      </c>
+      <c r="C10" s="20">
+        <v>1.746</v>
+      </c>
+      <c r="D10" s="20">
+        <v>2.4948999999999999</v>
+      </c>
+      <c r="E10" s="20">
+        <f t="shared" si="1"/>
+        <v>-0.7488999999999999</v>
+      </c>
+      <c r="F10" s="20">
+        <f>2*E10</f>
+        <v>-1.4977999999999998</v>
+      </c>
+      <c r="G10" s="19">
+        <v>-1.5</v>
+      </c>
+      <c r="H10" s="20">
+        <v>-1.4972000000000001</v>
+      </c>
+      <c r="I10" s="20">
+        <f t="shared" si="3"/>
+        <v>-2.7999999999999137E-3</v>
+      </c>
+      <c r="J10" s="19">
+        <f t="shared" si="0"/>
+        <v>0.18666666666666093</v>
+      </c>
+      <c r="K10" s="19">
+        <v>2.0230000000000001</v>
+      </c>
+      <c r="L10" s="21">
+        <v>3.9929999999999999</v>
+      </c>
+      <c r="M10" s="21">
+        <v>2.4956999999999998</v>
+      </c>
+    </row>
+    <row r="11" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B11" s="19">
+        <v>-25</v>
+      </c>
+      <c r="C11" s="20">
+        <v>1.8712</v>
+      </c>
+      <c r="D11" s="20">
+        <v>2.4948999999999999</v>
+      </c>
+      <c r="E11" s="20">
+        <f t="shared" si="1"/>
+        <v>-0.62369999999999992</v>
+      </c>
+      <c r="F11" s="20">
+        <f t="shared" si="2"/>
+        <v>-1.2473999999999998</v>
+      </c>
+      <c r="G11" s="19">
+        <v>-1.25</v>
+      </c>
+      <c r="H11" s="20">
+        <v>-1.2475000000000001</v>
+      </c>
+      <c r="I11" s="20">
+        <f t="shared" si="3"/>
+        <v>-2.4999999999999467E-3</v>
+      </c>
+      <c r="J11" s="19">
+        <f t="shared" si="0"/>
+        <v>0.19999999999999576</v>
+      </c>
+      <c r="K11" s="19">
+        <v>2.0270000000000001</v>
+      </c>
+      <c r="L11" s="21">
+        <v>3.7433000000000001</v>
+      </c>
+      <c r="M11" s="21">
+        <v>2.4956999999999998</v>
+      </c>
+    </row>
+    <row r="12" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B12" s="19">
+        <v>-20</v>
+      </c>
+      <c r="C12" s="20">
+        <v>1.996</v>
+      </c>
+      <c r="D12" s="20">
+        <v>2.4948999999999999</v>
+      </c>
+      <c r="E12" s="20">
+        <f t="shared" si="1"/>
+        <v>-0.4988999999999999</v>
+      </c>
+      <c r="F12" s="20">
+        <f t="shared" si="2"/>
+        <v>-0.9977999999999998</v>
+      </c>
+      <c r="G12" s="19">
+        <v>-1</v>
+      </c>
+      <c r="H12" s="20">
+        <v>-0.99809999999999999</v>
+      </c>
+      <c r="I12" s="20">
+        <f t="shared" si="3"/>
+        <v>-1.9000000000000128E-3</v>
+      </c>
+      <c r="J12" s="19">
+        <f t="shared" si="0"/>
+        <v>0.19000000000000128</v>
+      </c>
+      <c r="K12" s="19"/>
+      <c r="L12" s="21"/>
+      <c r="M12" s="21"/>
+    </row>
+    <row r="13" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B13" s="19">
+        <v>-15</v>
+      </c>
+      <c r="C13" s="20">
+        <v>2.1202000000000001</v>
+      </c>
+      <c r="D13" s="20">
+        <v>2.4950999999999999</v>
+      </c>
+      <c r="E13" s="20">
+        <f t="shared" si="1"/>
+        <v>-0.37489999999999979</v>
+      </c>
+      <c r="F13" s="20">
+        <f t="shared" si="2"/>
+        <v>-0.74979999999999958</v>
+      </c>
+      <c r="G13" s="19">
+        <v>-0.75</v>
+      </c>
+      <c r="H13" s="20">
+        <v>-0.75029999999999997</v>
+      </c>
+      <c r="I13" s="20">
+        <f t="shared" si="3"/>
+        <v>2.9999999999996696E-4</v>
+      </c>
+      <c r="J13" s="19">
+        <f t="shared" si="0"/>
+        <v>-3.9999999999995595E-2</v>
+      </c>
+      <c r="K13" s="19"/>
+      <c r="L13" s="21"/>
+      <c r="M13" s="21"/>
+    </row>
+    <row r="14" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B14" s="19">
+        <v>-10</v>
+      </c>
+      <c r="C14" s="20">
+        <v>2.242</v>
+      </c>
+      <c r="D14" s="20">
+        <v>2.4942000000000002</v>
+      </c>
+      <c r="E14" s="20">
+        <f t="shared" si="1"/>
+        <v>-0.2522000000000002</v>
+      </c>
+      <c r="F14" s="20">
+        <f t="shared" si="2"/>
+        <v>-0.5044000000000004</v>
+      </c>
+      <c r="G14" s="19">
+        <v>-0.5</v>
+      </c>
+      <c r="H14" s="20">
+        <v>-0.50439999999999996</v>
+      </c>
+      <c r="I14" s="20">
+        <f t="shared" ref="I14:I24" si="4">G14-H14</f>
+        <v>4.3999999999999595E-3</v>
+      </c>
+      <c r="J14" s="19">
+        <f t="shared" ref="J14:J24" si="5">(I14/G14)*100</f>
+        <v>-0.8799999999999919</v>
+      </c>
+      <c r="K14" s="19">
+        <v>2.0339999999999998</v>
+      </c>
+      <c r="L14" s="21">
+        <v>2.9940000000000002</v>
+      </c>
+      <c r="M14" s="21">
+        <v>2.4950999999999999</v>
+      </c>
+    </row>
+    <row r="15" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B15" s="19">
+        <v>-8</v>
+      </c>
+      <c r="C15" s="20">
+        <v>2.2919999999999998</v>
+      </c>
+      <c r="D15" s="20">
+        <v>2.4941</v>
+      </c>
+      <c r="E15" s="20">
+        <f t="shared" si="1"/>
+        <v>-0.20210000000000017</v>
+      </c>
+      <c r="F15" s="20">
+        <f t="shared" si="2"/>
+        <v>-0.40420000000000034</v>
+      </c>
+      <c r="G15" s="19">
+        <v>-0.4</v>
+      </c>
+      <c r="H15" s="20">
+        <v>-0.40425</v>
+      </c>
+      <c r="I15" s="20">
+        <f t="shared" si="4"/>
+        <v>4.249999999999976E-3</v>
+      </c>
+      <c r="J15" s="19">
+        <f t="shared" si="5"/>
+        <v>-1.062499999999994</v>
+      </c>
+      <c r="K15" s="19"/>
+      <c r="L15" s="21"/>
+      <c r="M15" s="21"/>
+    </row>
+    <row r="16" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B16" s="19">
+        <v>-6</v>
+      </c>
+      <c r="C16" s="20">
+        <v>2.3420000000000001</v>
+      </c>
+      <c r="D16" s="20">
+        <v>2.4941</v>
+      </c>
+      <c r="E16" s="20">
+        <f t="shared" si="1"/>
+        <v>-0.1520999999999999</v>
+      </c>
+      <c r="F16" s="20">
+        <f t="shared" si="2"/>
+        <v>-0.3041999999999998</v>
+      </c>
+      <c r="G16" s="19">
+        <v>-0.3</v>
+      </c>
+      <c r="H16" s="20">
+        <v>-0.30413000000000001</v>
+      </c>
+      <c r="I16" s="20">
+        <f t="shared" si="4"/>
+        <v>4.1300000000000225E-3</v>
+      </c>
+      <c r="J16" s="19">
+        <f t="shared" si="5"/>
+        <v>-1.3766666666666743</v>
+      </c>
+      <c r="K16" s="19"/>
+      <c r="L16" s="21"/>
+      <c r="M16" s="21"/>
+    </row>
+    <row r="17" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B17" s="19">
+        <v>-4</v>
+      </c>
+      <c r="C17" s="20">
+        <v>2.3919999999999999</v>
+      </c>
+      <c r="D17" s="20">
+        <v>2.4941</v>
+      </c>
+      <c r="E17" s="20">
+        <f t="shared" si="1"/>
+        <v>-0.10210000000000008</v>
+      </c>
+      <c r="F17" s="20">
+        <f t="shared" si="2"/>
+        <v>-0.20420000000000016</v>
+      </c>
+      <c r="G17" s="19">
+        <v>-0.2</v>
+      </c>
+      <c r="H17" s="20">
+        <v>-0.20399999999999999</v>
+      </c>
+      <c r="I17" s="20">
+        <f t="shared" si="4"/>
+        <v>3.9999999999999758E-3</v>
+      </c>
+      <c r="J17" s="19">
+        <f t="shared" si="5"/>
+        <v>-1.999999999999988</v>
+      </c>
+      <c r="K17" s="19"/>
+      <c r="L17" s="21"/>
+      <c r="M17" s="21"/>
+    </row>
+    <row r="18" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B18" s="19">
+        <v>-2</v>
+      </c>
+      <c r="C18" s="20">
+        <v>2.4420999999999999</v>
+      </c>
+      <c r="D18" s="20">
+        <v>2.4940000000000002</v>
+      </c>
+      <c r="E18" s="20">
+        <f t="shared" si="1"/>
+        <v>-5.1900000000000279E-2</v>
+      </c>
+      <c r="F18" s="20">
+        <f t="shared" si="2"/>
+        <v>-0.10380000000000056</v>
+      </c>
+      <c r="G18" s="19">
+        <v>-0.1</v>
+      </c>
+      <c r="H18" s="20">
+        <v>-0.104</v>
+      </c>
+      <c r="I18" s="20">
+        <f t="shared" si="4"/>
+        <v>3.9999999999999897E-3</v>
+      </c>
+      <c r="J18" s="19">
+        <f t="shared" si="5"/>
+        <v>-3.9999999999999898</v>
+      </c>
+      <c r="K18" s="19"/>
+      <c r="L18" s="21"/>
+      <c r="M18" s="21"/>
+    </row>
+    <row r="19" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B19" s="19">
+        <v>0</v>
+      </c>
+      <c r="C19" s="20">
+        <v>2.492</v>
+      </c>
+      <c r="D19" s="20">
+        <v>2.4940000000000002</v>
+      </c>
+      <c r="E19" s="20">
+        <f t="shared" si="1"/>
+        <v>-2.0000000000002238E-3</v>
+      </c>
+      <c r="F19" s="20">
+        <f t="shared" si="2"/>
+        <v>-4.0000000000004476E-3</v>
+      </c>
+      <c r="G19" s="19">
+        <v>0</v>
+      </c>
+      <c r="H19" s="20">
+        <v>-4.3E-3</v>
+      </c>
+      <c r="I19" s="20">
+        <f t="shared" si="4"/>
+        <v>4.3E-3</v>
+      </c>
+      <c r="J19" s="19" t="e">
+        <f t="shared" si="5"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="K19" s="19">
+        <v>2.0394000000000001</v>
+      </c>
+      <c r="L19" s="19">
+        <v>2.5</v>
+      </c>
+      <c r="M19" s="19">
+        <v>2.4948000000000001</v>
+      </c>
+    </row>
+    <row r="20" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B20" s="19">
+        <v>2</v>
+      </c>
+      <c r="C20" s="20">
+        <v>2.5423</v>
+      </c>
+      <c r="D20" s="20">
+        <v>2.4940000000000002</v>
+      </c>
+      <c r="E20" s="20">
+        <f t="shared" si="1"/>
+        <v>4.8299999999999788E-2</v>
+      </c>
+      <c r="F20" s="20">
+        <f t="shared" si="2"/>
+        <v>9.6599999999999575E-2</v>
+      </c>
+      <c r="G20" s="19">
+        <v>0.1</v>
+      </c>
+      <c r="H20" s="20">
+        <v>9.6299999999999997E-2</v>
+      </c>
+      <c r="I20" s="20">
+        <f t="shared" si="4"/>
+        <v>3.7000000000000088E-3</v>
+      </c>
+      <c r="J20" s="19">
+        <f t="shared" si="5"/>
+        <v>3.7000000000000091</v>
+      </c>
+      <c r="K20" s="19"/>
+      <c r="L20" s="21"/>
+      <c r="M20" s="21"/>
+    </row>
+    <row r="21" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B21" s="19">
+        <v>4</v>
+      </c>
+      <c r="C21" s="20">
+        <v>2.5920999999999998</v>
+      </c>
+      <c r="D21" s="20">
+        <v>2.4940000000000002</v>
+      </c>
+      <c r="E21" s="20">
+        <f t="shared" si="1"/>
+        <v>9.8099999999999632E-2</v>
+      </c>
+      <c r="F21" s="20">
+        <f t="shared" si="2"/>
+        <v>0.19619999999999926</v>
+      </c>
+      <c r="G21" s="19">
+        <v>0.2</v>
+      </c>
+      <c r="H21" s="20">
+        <v>0.19639999999999999</v>
+      </c>
+      <c r="I21" s="20">
+        <f t="shared" si="4"/>
+        <v>3.6000000000000199E-3</v>
+      </c>
+      <c r="J21" s="19">
+        <f t="shared" si="5"/>
+        <v>1.80000000000001</v>
+      </c>
+      <c r="K21" s="19"/>
+      <c r="L21" s="21"/>
+      <c r="M21" s="21"/>
+    </row>
+    <row r="22" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B22" s="19">
+        <v>6</v>
+      </c>
+      <c r="C22" s="20">
+        <v>2.6419999999999999</v>
+      </c>
+      <c r="D22" s="20">
+        <v>2.4941</v>
+      </c>
+      <c r="E22" s="20">
+        <f t="shared" si="1"/>
+        <v>0.14789999999999992</v>
+      </c>
+      <c r="F22" s="20">
+        <f t="shared" si="2"/>
+        <v>0.29579999999999984</v>
+      </c>
+      <c r="G22" s="19">
+        <v>0.3</v>
+      </c>
+      <c r="H22" s="20">
+        <v>0.29620000000000002</v>
+      </c>
+      <c r="I22" s="20">
+        <f t="shared" si="4"/>
+        <v>3.7999999999999701E-3</v>
+      </c>
+      <c r="J22" s="19">
+        <f t="shared" si="5"/>
+        <v>1.2666666666666568</v>
+      </c>
+      <c r="K22" s="19"/>
+      <c r="L22" s="21"/>
+      <c r="M22" s="21"/>
+    </row>
+    <row r="23" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B23" s="19">
+        <v>8</v>
+      </c>
+      <c r="C23" s="20">
+        <v>2.6920000000000002</v>
+      </c>
+      <c r="D23" s="20">
+        <v>2.4941</v>
+      </c>
+      <c r="E23" s="20">
+        <f t="shared" si="1"/>
+        <v>0.19790000000000019</v>
+      </c>
+      <c r="F23" s="20">
+        <f t="shared" si="2"/>
+        <v>0.39580000000000037</v>
+      </c>
+      <c r="G23" s="19">
+        <v>0.4</v>
+      </c>
+      <c r="H23" s="20">
+        <v>0.39600000000000002</v>
+      </c>
+      <c r="I23" s="20">
+        <f t="shared" si="4"/>
+        <v>4.0000000000000036E-3</v>
+      </c>
+      <c r="J23" s="19">
+        <f t="shared" si="5"/>
+        <v>1.0000000000000009</v>
+      </c>
+      <c r="K23" s="19"/>
+      <c r="L23" s="21"/>
+      <c r="M23" s="21"/>
+    </row>
+    <row r="24" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B24" s="19">
+        <v>10</v>
+      </c>
+      <c r="C24" s="20">
+        <v>2.7421000000000002</v>
+      </c>
+      <c r="D24" s="20">
+        <v>2.4941</v>
+      </c>
+      <c r="E24" s="20">
+        <f t="shared" si="1"/>
+        <v>0.24800000000000022</v>
+      </c>
+      <c r="F24" s="20">
+        <f t="shared" si="2"/>
+        <v>0.49600000000000044</v>
+      </c>
+      <c r="G24" s="19">
+        <v>0.5</v>
+      </c>
+      <c r="H24" s="20">
+        <v>0.49569999999999997</v>
+      </c>
+      <c r="I24" s="20">
+        <f t="shared" si="4"/>
+        <v>4.300000000000026E-3</v>
+      </c>
+      <c r="J24" s="19">
+        <f t="shared" si="5"/>
+        <v>0.8600000000000052</v>
+      </c>
+      <c r="K24" s="19">
+        <v>2.0394000000000001</v>
+      </c>
+      <c r="L24" s="21"/>
+      <c r="M24" s="21"/>
+    </row>
+    <row r="25" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B25" s="19">
+        <v>15</v>
+      </c>
+      <c r="C25" s="19">
+        <v>2.8650000000000002</v>
+      </c>
+      <c r="D25" s="20">
+        <v>2.4942000000000002</v>
+      </c>
+      <c r="E25" s="20">
+        <f t="shared" si="1"/>
+        <v>0.37080000000000002</v>
+      </c>
+      <c r="F25" s="20">
+        <f t="shared" si="2"/>
+        <v>0.74160000000000004</v>
+      </c>
+      <c r="G25" s="19">
+        <v>0.75</v>
+      </c>
+      <c r="H25" s="19">
+        <v>0.74180000000000001</v>
+      </c>
+      <c r="I25" s="20">
+        <f t="shared" ref="I25:I32" si="6">G25-H25</f>
+        <v>8.1999999999999851E-3</v>
+      </c>
+      <c r="J25" s="19">
+        <f t="shared" ref="J25:J32" si="7">(I25/G25)*100</f>
+        <v>1.0933333333333315</v>
+      </c>
+      <c r="K25" s="19"/>
+      <c r="L25" s="21"/>
+      <c r="M25" s="21"/>
+    </row>
+    <row r="26" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B26" s="19">
+        <v>20</v>
+      </c>
+      <c r="C26" s="19">
+        <v>2.9889999999999999</v>
+      </c>
+      <c r="D26" s="20">
+        <v>2.4942000000000002</v>
+      </c>
+      <c r="E26" s="20">
+        <f t="shared" si="1"/>
+        <v>0.49479999999999968</v>
+      </c>
+      <c r="F26" s="20">
+        <f t="shared" si="2"/>
+        <v>0.98959999999999937</v>
+      </c>
+      <c r="G26" s="19">
+        <v>1</v>
+      </c>
+      <c r="H26" s="19">
+        <v>0.98929999999999996</v>
+      </c>
+      <c r="I26" s="20">
+        <f t="shared" si="6"/>
+        <v>1.0700000000000043E-2</v>
+      </c>
+      <c r="J26" s="19">
+        <f t="shared" si="7"/>
+        <v>1.0700000000000043</v>
+      </c>
+      <c r="K26" s="19"/>
+      <c r="L26" s="21"/>
+      <c r="M26" s="21"/>
+    </row>
+    <row r="27" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B27" s="19">
+        <v>25</v>
+      </c>
+      <c r="C27" s="19">
+        <v>3.1135000000000002</v>
+      </c>
+      <c r="D27" s="20">
+        <v>2.4943</v>
+      </c>
+      <c r="E27" s="20">
+        <f t="shared" si="1"/>
+        <v>0.61920000000000019</v>
+      </c>
+      <c r="F27" s="20">
+        <f t="shared" si="2"/>
+        <v>1.2384000000000004</v>
+      </c>
+      <c r="G27" s="19">
+        <v>1.25</v>
+      </c>
+      <c r="H27" s="19">
+        <v>1.2370000000000001</v>
+      </c>
+      <c r="I27" s="20">
+        <f t="shared" si="6"/>
+        <v>1.2999999999999901E-2</v>
+      </c>
+      <c r="J27" s="19">
+        <f t="shared" si="7"/>
+        <v>1.039999999999992</v>
+      </c>
+      <c r="K27" s="19">
+        <v>2.0390000000000001</v>
+      </c>
+      <c r="L27" s="21"/>
+      <c r="M27" s="21"/>
+    </row>
+    <row r="28" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B28" s="19">
+        <v>30</v>
+      </c>
+      <c r="C28" s="19">
+        <v>3.2389999999999999</v>
+      </c>
+      <c r="D28" s="20">
+        <v>2.4946000000000002</v>
+      </c>
+      <c r="E28" s="20">
+        <f t="shared" si="1"/>
+        <v>0.74439999999999973</v>
+      </c>
+      <c r="F28" s="20">
+        <f t="shared" si="2"/>
+        <v>1.4887999999999995</v>
+      </c>
+      <c r="G28" s="19">
+        <v>1.5</v>
+      </c>
+      <c r="H28" s="19">
+        <v>1.4883</v>
+      </c>
+      <c r="I28" s="20">
+        <f t="shared" si="6"/>
+        <v>1.1700000000000044E-2</v>
+      </c>
+      <c r="J28" s="19">
+        <f t="shared" si="7"/>
+        <v>0.78000000000000291</v>
+      </c>
+      <c r="K28" s="19"/>
+      <c r="L28" s="21"/>
+      <c r="M28" s="21"/>
+    </row>
+    <row r="29" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B29" s="19">
+        <v>35</v>
+      </c>
+      <c r="C29" s="19">
+        <v>3.3639999999999999</v>
+      </c>
+      <c r="D29" s="20">
+        <v>2.4946999999999999</v>
+      </c>
+      <c r="E29" s="20">
+        <f t="shared" si="1"/>
+        <v>0.86929999999999996</v>
+      </c>
+      <c r="F29" s="20">
+        <f t="shared" si="2"/>
+        <v>1.7385999999999999</v>
+      </c>
+      <c r="G29" s="19">
+        <v>1.75</v>
+      </c>
+      <c r="H29" s="19">
+        <v>1.7378</v>
+      </c>
+      <c r="I29" s="20">
+        <f t="shared" si="6"/>
+        <v>1.2199999999999989E-2</v>
+      </c>
+      <c r="J29" s="19">
+        <f t="shared" si="7"/>
+        <v>0.69714285714285651</v>
+      </c>
+      <c r="K29" s="19"/>
+      <c r="L29" s="21"/>
+      <c r="M29" s="21"/>
+    </row>
+    <row r="30" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B30" s="19">
+        <v>40</v>
+      </c>
+      <c r="C30" s="19">
+        <v>3.4891999999999999</v>
+      </c>
+      <c r="D30" s="20">
+        <v>2.4948999999999999</v>
+      </c>
+      <c r="E30" s="20">
+        <f t="shared" si="1"/>
+        <v>0.99429999999999996</v>
+      </c>
+      <c r="F30" s="20">
+        <f t="shared" si="2"/>
+        <v>1.9885999999999999</v>
+      </c>
+      <c r="G30" s="19">
+        <v>2</v>
+      </c>
+      <c r="H30" s="19">
+        <v>1.9884999999999999</v>
+      </c>
+      <c r="I30" s="20">
+        <f t="shared" si="6"/>
+        <v>1.1500000000000066E-2</v>
+      </c>
+      <c r="J30" s="19">
+        <f t="shared" si="7"/>
+        <v>0.57500000000000329</v>
+      </c>
+      <c r="K30" s="19">
+        <v>2.0299999999999998</v>
+      </c>
+      <c r="L30" s="21"/>
+      <c r="M30" s="21"/>
+    </row>
+    <row r="31" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B31" s="19">
+        <v>45</v>
+      </c>
+      <c r="C31" s="19">
+        <v>3.6145</v>
+      </c>
+      <c r="D31" s="20">
+        <v>2.4950000000000001</v>
+      </c>
+      <c r="E31" s="20">
+        <f t="shared" si="1"/>
+        <v>1.1194999999999999</v>
+      </c>
+      <c r="F31" s="20">
+        <f t="shared" si="2"/>
+        <v>2.2389999999999999</v>
+      </c>
+      <c r="G31" s="19">
+        <v>2.25</v>
+      </c>
+      <c r="H31" s="19">
+        <v>2.2385000000000002</v>
+      </c>
+      <c r="I31" s="20">
+        <f t="shared" si="6"/>
+        <v>1.1499999999999844E-2</v>
+      </c>
+      <c r="J31" s="19">
+        <f t="shared" si="7"/>
+        <v>0.51111111111110419</v>
+      </c>
+      <c r="K31" s="19"/>
+      <c r="L31" s="21"/>
+      <c r="M31" s="21"/>
+    </row>
+    <row r="32" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B32" s="19">
+        <v>50</v>
+      </c>
+      <c r="C32" s="19">
+        <v>3.7397</v>
+      </c>
+      <c r="D32" s="20">
+        <v>2.4952000000000001</v>
+      </c>
+      <c r="E32" s="20">
+        <f t="shared" si="1"/>
+        <v>1.2444999999999999</v>
+      </c>
+      <c r="F32" s="20">
+        <f t="shared" si="2"/>
+        <v>2.4889999999999999</v>
+      </c>
+      <c r="G32" s="19">
+        <v>2.5</v>
+      </c>
+      <c r="H32" s="19">
+        <v>2.4731999999999998</v>
+      </c>
+      <c r="I32" s="20">
+        <f t="shared" si="6"/>
+        <v>2.6800000000000157E-2</v>
+      </c>
+      <c r="J32" s="19">
+        <f t="shared" si="7"/>
+        <v>1.0720000000000063</v>
+      </c>
+      <c r="K32" s="19">
+        <v>2.02</v>
+      </c>
+      <c r="L32" s="21"/>
+      <c r="M32" s="21"/>
+    </row>
+    <row r="33" spans="2:13" s="22" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B33" s="23"/>
+      <c r="C33" s="23"/>
+      <c r="D33" s="23"/>
+      <c r="E33" s="23"/>
+      <c r="F33" s="23"/>
+      <c r="G33" s="24"/>
+      <c r="H33" s="23"/>
+      <c r="I33" s="23"/>
+      <c r="J33" s="23"/>
+      <c r="K33" s="23"/>
+      <c r="L33" s="23"/>
+      <c r="M33" s="23"/>
+    </row>
+    <row r="34" spans="2:13" s="22" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B34" s="23"/>
+      <c r="C34" s="23"/>
+      <c r="D34" s="23"/>
+      <c r="E34" s="23"/>
+      <c r="F34" s="23"/>
+      <c r="G34" s="24"/>
+      <c r="H34" s="23"/>
+      <c r="I34" s="23"/>
+      <c r="J34" s="23"/>
+      <c r="K34" s="23"/>
+      <c r="L34" s="23"/>
+      <c r="M34" s="23"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1B0A327-0A3E-402F-85E2-FF0CDB51D013}">
+  <dimension ref="B1:L19"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="3" max="3" width="16.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.6328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.6328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.36328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.6328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.54296875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:12" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="B1" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1" s="12"/>
+    </row>
+    <row r="4" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B4" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="18" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="17" t="s">
+        <v>1</v>
+      </c>
+      <c r="F4" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="H4" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="I4" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="J4" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="K4" s="17" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="5" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B5" s="19">
+        <v>-50</v>
+      </c>
+      <c r="C5" s="20">
+        <v>1.2462</v>
+      </c>
+      <c r="D5" s="20">
+        <v>2.4950999999999999</v>
+      </c>
+      <c r="E5" s="20">
+        <f>C5-D5</f>
+        <v>-1.2488999999999999</v>
+      </c>
+      <c r="F5" s="20">
+        <f>2*E5</f>
+        <v>-2.4977999999999998</v>
+      </c>
+      <c r="G5" s="19">
+        <v>-2.5</v>
+      </c>
+      <c r="H5" s="20">
+        <v>-2.3965999999999998</v>
+      </c>
+      <c r="I5" s="20">
+        <f>G5-H5</f>
+        <v>-0.10340000000000016</v>
+      </c>
+      <c r="J5" s="19">
+        <f t="shared" ref="J5:J13" si="0">(I5/G5)*100</f>
+        <v>4.1360000000000063</v>
+      </c>
+      <c r="K5" s="19">
+        <v>2.0084</v>
+      </c>
+      <c r="L5" s="14"/>
+    </row>
+    <row r="6" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B6" s="19">
+        <v>-45</v>
+      </c>
+      <c r="C6" s="20">
+        <v>1.3712</v>
+      </c>
+      <c r="D6" s="20">
+        <v>2.4950000000000001</v>
+      </c>
+      <c r="E6" s="20">
+        <f t="shared" ref="E6:E13" si="1">C6-D6</f>
+        <v>-1.1238000000000001</v>
+      </c>
+      <c r="F6" s="20">
+        <f t="shared" ref="F6:F8" si="2">2*E6</f>
+        <v>-2.2476000000000003</v>
+      </c>
+      <c r="G6" s="19">
+        <v>-2.25</v>
+      </c>
+      <c r="H6" s="20">
+        <v>-2.1551999999999998</v>
+      </c>
+      <c r="I6" s="20">
+        <f t="shared" ref="I6:I13" si="3">G6-H6</f>
+        <v>-9.4800000000000217E-2</v>
+      </c>
+      <c r="J6" s="19">
+        <f t="shared" si="0"/>
+        <v>4.2133333333333436</v>
+      </c>
+      <c r="K6" s="19">
+        <v>2.0084</v>
+      </c>
+    </row>
+    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B7" s="19">
+        <v>-40</v>
+      </c>
+      <c r="C7" s="20">
+        <v>1.4961</v>
+      </c>
+      <c r="D7" s="20">
+        <v>2.4950000000000001</v>
+      </c>
+      <c r="E7" s="20">
+        <f t="shared" si="1"/>
+        <v>-0.99890000000000012</v>
+      </c>
+      <c r="F7" s="20">
+        <f t="shared" si="2"/>
+        <v>-1.9978000000000002</v>
+      </c>
+      <c r="G7" s="19">
+        <v>-2</v>
+      </c>
+      <c r="H7" s="20">
+        <v>-1.915</v>
+      </c>
+      <c r="I7" s="20">
+        <f t="shared" si="3"/>
+        <v>-8.4999999999999964E-2</v>
+      </c>
+      <c r="J7" s="19">
+        <f t="shared" si="0"/>
+        <v>4.2499999999999982</v>
+      </c>
+      <c r="K7" s="19">
+        <v>2.0087999999999999</v>
+      </c>
+    </row>
+    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B8" s="19">
+        <v>-35</v>
+      </c>
+      <c r="C8" s="20">
+        <v>1.6212</v>
+      </c>
+      <c r="D8" s="20">
+        <v>2.4948999999999999</v>
+      </c>
+      <c r="E8" s="20">
         <f t="shared" si="1"/>
         <v>-0.87369999999999992</v>
       </c>
-      <c r="F9" s="14">
+      <c r="F8" s="20">
         <f t="shared" si="2"/>
         <v>-1.7473999999999998</v>
       </c>
-      <c r="G9" s="13">
+      <c r="G8" s="19">
         <v>-1.75</v>
       </c>
-      <c r="H9" s="14">
-        <v>-1.5949</v>
-      </c>
-      <c r="I9" s="14">
+      <c r="H8" s="20">
+        <v>-1.6744000000000001</v>
+      </c>
+      <c r="I8" s="20">
         <f t="shared" si="3"/>
-        <v>-0.15510000000000002</v>
-      </c>
-      <c r="J9" s="13">
+        <v>-7.559999999999989E-2</v>
+      </c>
+      <c r="J8" s="19">
         <f t="shared" si="0"/>
-        <v>8.862857142857143</v>
-      </c>
-    </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B10" s="3">
+        <v>4.3199999999999941</v>
+      </c>
+      <c r="K8" s="19">
+        <v>2.0084</v>
+      </c>
+    </row>
+    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B9" s="19">
         <v>-30</v>
       </c>
-      <c r="C10" s="7">
+      <c r="C9" s="20">
         <v>1.746</v>
       </c>
-      <c r="D10" s="7">
+      <c r="D9" s="20">
         <v>2.4948999999999999</v>
       </c>
-      <c r="E10" s="7">
+      <c r="E9" s="20">
         <f t="shared" si="1"/>
         <v>-0.7488999999999999</v>
       </c>
-      <c r="F10" s="7">
-        <f>2*E10</f>
+      <c r="F9" s="20">
+        <f>2*E9</f>
         <v>-1.4977999999999998</v>
       </c>
-      <c r="G10" s="3">
+      <c r="G9" s="19">
         <v>-1.5</v>
       </c>
-      <c r="H10" s="7">
-        <v>-1.4972000000000001</v>
-      </c>
-      <c r="I10" s="7">
+      <c r="H9" s="20">
+        <v>-1.4372</v>
+      </c>
+      <c r="I9" s="20">
         <f t="shared" si="3"/>
-        <v>-2.7999999999999137E-3</v>
-      </c>
-      <c r="J10" s="3">
+        <v>-6.2799999999999967E-2</v>
+      </c>
+      <c r="J9" s="19">
         <f t="shared" si="0"/>
-        <v>0.18666666666666093</v>
-      </c>
-    </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B11" s="3">
-        <v>-25</v>
-      </c>
-      <c r="C11" s="7">
-        <v>1.8712</v>
-      </c>
-      <c r="D11" s="7">
-        <v>2.4948999999999999</v>
-      </c>
-      <c r="E11" s="7">
-        <f t="shared" si="1"/>
-        <v>-0.62369999999999992</v>
-      </c>
-      <c r="F11" s="7">
-        <f t="shared" si="2"/>
-        <v>-1.2473999999999998</v>
-      </c>
-      <c r="G11" s="3">
-        <v>-1.25</v>
-      </c>
-      <c r="H11" s="7">
-        <v>-1.2475000000000001</v>
-      </c>
-      <c r="I11" s="7">
-        <f t="shared" si="3"/>
-        <v>-2.4999999999999467E-3</v>
-      </c>
-      <c r="J11" s="3">
-        <f t="shared" si="0"/>
-        <v>0.19999999999999576</v>
-      </c>
-    </row>
-    <row r="12" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B12" s="3">
-        <v>-20</v>
-      </c>
-      <c r="C12" s="7">
-        <v>1.996</v>
-      </c>
-      <c r="D12" s="7">
-        <v>2.4948999999999999</v>
-      </c>
-      <c r="E12" s="7">
-        <f t="shared" si="1"/>
-        <v>-0.4988999999999999</v>
-      </c>
-      <c r="F12" s="7">
-        <f t="shared" si="2"/>
-        <v>-0.9977999999999998</v>
-      </c>
-      <c r="G12" s="3">
-        <v>-1</v>
-      </c>
-      <c r="H12" s="7">
-        <v>-0.99809999999999999</v>
-      </c>
-      <c r="I12" s="7">
-        <f t="shared" si="3"/>
-        <v>-1.9000000000000128E-3</v>
-      </c>
-      <c r="J12" s="3">
-        <f t="shared" si="0"/>
-        <v>0.19000000000000128</v>
-      </c>
-    </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B13" s="3">
-        <v>-15</v>
-      </c>
-      <c r="C13" s="7">
-        <v>2.1202000000000001</v>
-      </c>
-      <c r="D13" s="7">
-        <v>2.4950999999999999</v>
-      </c>
-      <c r="E13" s="7">
-        <f t="shared" si="1"/>
-        <v>-0.37489999999999979</v>
-      </c>
-      <c r="F13" s="7">
-        <f t="shared" si="2"/>
-        <v>-0.74979999999999958</v>
-      </c>
-      <c r="G13" s="3">
-        <v>-0.75</v>
-      </c>
-      <c r="H13" s="7">
-        <v>-0.75029999999999997</v>
-      </c>
-      <c r="I13" s="7">
-        <f t="shared" si="3"/>
-        <v>2.9999999999996696E-4</v>
-      </c>
-      <c r="J13" s="3">
-        <f t="shared" si="0"/>
-        <v>-3.9999999999995595E-2</v>
-      </c>
-    </row>
-    <row r="14" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B14" s="3">
-        <v>-10</v>
-      </c>
-      <c r="C14" s="7">
-        <v>2.242</v>
-      </c>
-      <c r="D14" s="7">
-        <v>2.4942000000000002</v>
-      </c>
-      <c r="E14" s="7">
-        <f t="shared" si="1"/>
-        <v>-0.2522000000000002</v>
-      </c>
-      <c r="F14" s="7">
-        <f t="shared" si="2"/>
-        <v>-0.5044000000000004</v>
-      </c>
-      <c r="G14" s="3">
-        <v>-0.5</v>
-      </c>
-      <c r="H14" s="7">
-        <v>-0.50439999999999996</v>
-      </c>
-      <c r="I14" s="7">
-        <f t="shared" ref="I14:I24" si="4">G14-H14</f>
-        <v>4.3999999999999595E-3</v>
-      </c>
-      <c r="J14" s="3">
-        <f t="shared" ref="J14:J24" si="5">(I14/G14)*100</f>
-        <v>-0.8799999999999919</v>
-      </c>
-    </row>
-    <row r="15" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B15" s="3">
-        <v>-8</v>
-      </c>
-      <c r="C15" s="7">
-        <v>2.2919999999999998</v>
-      </c>
-      <c r="D15" s="7">
-        <v>2.4941</v>
-      </c>
-      <c r="E15" s="7">
-        <f t="shared" si="1"/>
-        <v>-0.20210000000000017</v>
-      </c>
-      <c r="F15" s="7">
-        <f t="shared" si="2"/>
-        <v>-0.40420000000000034</v>
-      </c>
-      <c r="G15" s="3">
-        <v>-0.4</v>
-      </c>
-      <c r="H15" s="7">
-        <v>-0.40425</v>
-      </c>
-      <c r="I15" s="7">
-        <f t="shared" si="4"/>
-        <v>4.249999999999976E-3</v>
-      </c>
-      <c r="J15" s="3">
-        <f t="shared" si="5"/>
-        <v>-1.062499999999994</v>
-      </c>
-    </row>
-    <row r="16" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B16" s="3">
-        <v>-6</v>
-      </c>
-      <c r="C16" s="7">
-        <v>2.3420000000000001</v>
-      </c>
-      <c r="D16" s="7">
-        <v>2.4941</v>
-      </c>
-      <c r="E16" s="7">
-        <f t="shared" si="1"/>
-        <v>-0.1520999999999999</v>
-      </c>
-      <c r="F16" s="7">
-        <f t="shared" si="2"/>
-        <v>-0.3041999999999998</v>
-      </c>
-      <c r="G16" s="3">
-        <v>-0.3</v>
-      </c>
-      <c r="H16" s="7">
-        <v>-0.30413000000000001</v>
-      </c>
-      <c r="I16" s="7">
-        <f t="shared" si="4"/>
-        <v>4.1300000000000225E-3</v>
-      </c>
-      <c r="J16" s="3">
-        <f t="shared" si="5"/>
-        <v>-1.3766666666666743</v>
-      </c>
-    </row>
-    <row r="17" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B17" s="3">
-        <v>-4</v>
-      </c>
-      <c r="C17" s="7">
-        <v>2.3919999999999999</v>
-      </c>
-      <c r="D17" s="7">
-        <v>2.4941</v>
-      </c>
-      <c r="E17" s="7">
-        <f t="shared" si="1"/>
-        <v>-0.10210000000000008</v>
-      </c>
-      <c r="F17" s="7">
-        <f t="shared" si="2"/>
-        <v>-0.20420000000000016</v>
-      </c>
-      <c r="G17" s="3">
-        <v>-0.2</v>
-      </c>
-      <c r="H17" s="7">
-        <v>-0.20399999999999999</v>
-      </c>
-      <c r="I17" s="7">
-        <f t="shared" si="4"/>
-        <v>3.9999999999999758E-3</v>
-      </c>
-      <c r="J17" s="3">
-        <f t="shared" si="5"/>
-        <v>-1.999999999999988</v>
-      </c>
-    </row>
-    <row r="18" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B18" s="3">
-        <v>-2</v>
-      </c>
-      <c r="C18" s="7">
-        <v>2.4420999999999999</v>
-      </c>
-      <c r="D18" s="7">
-        <v>2.4940000000000002</v>
-      </c>
-      <c r="E18" s="7">
-        <f t="shared" si="1"/>
-        <v>-5.1900000000000279E-2</v>
-      </c>
-      <c r="F18" s="7">
-        <f t="shared" si="2"/>
-        <v>-0.10380000000000056</v>
-      </c>
-      <c r="G18" s="3">
-        <v>-0.1</v>
-      </c>
-      <c r="H18" s="7">
-        <v>-0.104</v>
-      </c>
-      <c r="I18" s="7">
-        <f t="shared" si="4"/>
-        <v>3.9999999999999897E-3</v>
-      </c>
-      <c r="J18" s="3">
-        <f t="shared" si="5"/>
-        <v>-3.9999999999999898</v>
-      </c>
-    </row>
-    <row r="19" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B19" s="3">
-        <v>0</v>
-      </c>
-      <c r="C19" s="7">
-        <v>2.492</v>
-      </c>
-      <c r="D19" s="7">
-        <v>2.4940000000000002</v>
-      </c>
-      <c r="E19" s="7">
-        <f t="shared" si="1"/>
-        <v>-2.0000000000002238E-3</v>
-      </c>
-      <c r="F19" s="7">
-        <f t="shared" si="2"/>
-        <v>-4.0000000000004476E-3</v>
-      </c>
-      <c r="G19" s="3">
-        <v>0</v>
-      </c>
-      <c r="H19" s="7">
-        <v>-4.3E-3</v>
-      </c>
-      <c r="I19" s="7">
-        <f t="shared" si="4"/>
-        <v>4.3E-3</v>
-      </c>
-      <c r="J19" s="3" t="e">
-        <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="20" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B20" s="3">
-        <v>2</v>
-      </c>
-      <c r="C20" s="7">
-        <v>2.5423</v>
-      </c>
-      <c r="D20" s="7">
-        <v>2.4940000000000002</v>
-      </c>
-      <c r="E20" s="7">
-        <f t="shared" si="1"/>
-        <v>4.8299999999999788E-2</v>
-      </c>
-      <c r="F20" s="7">
-        <f t="shared" si="2"/>
-        <v>9.6599999999999575E-2</v>
-      </c>
-      <c r="G20" s="3">
-        <v>0.1</v>
-      </c>
-      <c r="H20" s="7">
-        <v>9.6299999999999997E-2</v>
-      </c>
-      <c r="I20" s="7">
-        <f t="shared" si="4"/>
-        <v>3.7000000000000088E-3</v>
-      </c>
-      <c r="J20" s="3">
-        <f t="shared" si="5"/>
-        <v>3.7000000000000091</v>
-      </c>
-    </row>
-    <row r="21" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B21" s="3">
-        <v>4</v>
-      </c>
-      <c r="C21" s="7">
-        <v>2.5920999999999998</v>
-      </c>
-      <c r="D21" s="7">
-        <v>2.4940000000000002</v>
-      </c>
-      <c r="E21" s="7">
-        <f t="shared" si="1"/>
-        <v>9.8099999999999632E-2</v>
-      </c>
-      <c r="F21" s="7">
-        <f t="shared" si="2"/>
-        <v>0.19619999999999926</v>
-      </c>
-      <c r="G21" s="3">
-        <v>0.2</v>
-      </c>
-      <c r="H21" s="7">
-        <v>0.19639999999999999</v>
-      </c>
-      <c r="I21" s="7">
-        <f t="shared" si="4"/>
-        <v>3.6000000000000199E-3</v>
-      </c>
-      <c r="J21" s="3">
-        <f t="shared" si="5"/>
-        <v>1.80000000000001</v>
-      </c>
-    </row>
-    <row r="22" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B22" s="3">
-        <v>6</v>
-      </c>
-      <c r="C22" s="7">
-        <v>2.6419999999999999</v>
-      </c>
-      <c r="D22" s="7">
-        <v>2.4941</v>
-      </c>
-      <c r="E22" s="7">
-        <f t="shared" si="1"/>
-        <v>0.14789999999999992</v>
-      </c>
-      <c r="F22" s="7">
-        <f t="shared" si="2"/>
-        <v>0.29579999999999984</v>
-      </c>
-      <c r="G22" s="3">
-        <v>0.3</v>
-      </c>
-      <c r="H22" s="7">
-        <v>0.29620000000000002</v>
-      </c>
-      <c r="I22" s="7">
-        <f t="shared" si="4"/>
-        <v>3.7999999999999701E-3</v>
-      </c>
-      <c r="J22" s="3">
-        <f t="shared" si="5"/>
-        <v>1.2666666666666568</v>
-      </c>
-    </row>
-    <row r="23" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B23" s="3">
-        <v>8</v>
-      </c>
-      <c r="C23" s="7">
-        <v>2.6920000000000002</v>
-      </c>
-      <c r="D23" s="7">
-        <v>2.4941</v>
-      </c>
-      <c r="E23" s="7">
-        <f t="shared" si="1"/>
-        <v>0.19790000000000019</v>
-      </c>
-      <c r="F23" s="7">
-        <f t="shared" si="2"/>
-        <v>0.39580000000000037</v>
-      </c>
-      <c r="G23" s="3">
-        <v>0.4</v>
-      </c>
-      <c r="H23" s="7">
-        <v>0.39600000000000002</v>
-      </c>
-      <c r="I23" s="7">
-        <f t="shared" si="4"/>
-        <v>4.0000000000000036E-3</v>
-      </c>
-      <c r="J23" s="3">
-        <f t="shared" si="5"/>
-        <v>1.0000000000000009</v>
-      </c>
-    </row>
-    <row r="24" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B24" s="3">
-        <v>10</v>
-      </c>
-      <c r="C24" s="7">
-        <v>2.7421000000000002</v>
-      </c>
-      <c r="D24" s="7">
-        <v>2.4941</v>
-      </c>
-      <c r="E24" s="7">
-        <f t="shared" si="1"/>
-        <v>0.24800000000000022</v>
-      </c>
-      <c r="F24" s="7">
-        <f t="shared" si="2"/>
-        <v>0.49600000000000044</v>
-      </c>
-      <c r="G24" s="3">
-        <v>0.5</v>
-      </c>
-      <c r="H24" s="7">
-        <v>0.49569999999999997</v>
-      </c>
-      <c r="I24" s="7">
-        <f t="shared" si="4"/>
-        <v>4.300000000000026E-3</v>
-      </c>
-      <c r="J24" s="3">
-        <f t="shared" si="5"/>
-        <v>0.8600000000000052</v>
-      </c>
-    </row>
-    <row r="25" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B25" s="3">
-        <v>15</v>
-      </c>
-      <c r="C25" s="3">
-        <v>2.8650000000000002</v>
-      </c>
-      <c r="D25" s="7">
-        <v>2.4942000000000002</v>
-      </c>
-      <c r="E25" s="7">
-        <f t="shared" si="1"/>
-        <v>0.37080000000000002</v>
-      </c>
-      <c r="F25" s="7">
-        <f t="shared" si="2"/>
-        <v>0.74160000000000004</v>
-      </c>
-      <c r="G25" s="3">
-        <v>0.75</v>
-      </c>
-      <c r="H25" s="3">
-        <v>0.74180000000000001</v>
-      </c>
-      <c r="I25" s="7">
-        <f t="shared" ref="I25:I32" si="6">G25-H25</f>
-        <v>8.1999999999999851E-3</v>
-      </c>
-      <c r="J25" s="3">
-        <f t="shared" ref="J25:J32" si="7">(I25/G25)*100</f>
-        <v>1.0933333333333315</v>
-      </c>
-    </row>
-    <row r="26" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B26" s="3">
-        <v>20</v>
-      </c>
-      <c r="C26" s="3">
-        <v>2.9889999999999999</v>
-      </c>
-      <c r="D26" s="7">
-        <v>2.4942000000000002</v>
-      </c>
-      <c r="E26" s="7">
-        <f t="shared" si="1"/>
-        <v>0.49479999999999968</v>
-      </c>
-      <c r="F26" s="7">
-        <f t="shared" si="2"/>
-        <v>0.98959999999999937</v>
-      </c>
-      <c r="G26" s="3">
-        <v>1</v>
-      </c>
-      <c r="H26" s="3">
-        <v>0.98929999999999996</v>
-      </c>
-      <c r="I26" s="7">
-        <f t="shared" si="6"/>
-        <v>1.0700000000000043E-2</v>
-      </c>
-      <c r="J26" s="3">
-        <f t="shared" si="7"/>
-        <v>1.0700000000000043</v>
-      </c>
-    </row>
-    <row r="27" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B27" s="3">
-        <v>25</v>
-      </c>
-      <c r="C27" s="3">
-        <v>3.1135000000000002</v>
-      </c>
-      <c r="D27" s="7">
-        <v>2.4943</v>
-      </c>
-      <c r="E27" s="7">
-        <f t="shared" si="1"/>
-        <v>0.61920000000000019</v>
-      </c>
-      <c r="F27" s="7">
-        <f t="shared" si="2"/>
-        <v>1.2384000000000004</v>
-      </c>
-      <c r="G27" s="3">
-        <v>1.25</v>
-      </c>
-      <c r="H27" s="3">
-        <v>1.2382</v>
-      </c>
-      <c r="I27" s="7">
-        <f t="shared" si="6"/>
-        <v>1.1800000000000033E-2</v>
-      </c>
-      <c r="J27" s="3">
-        <f t="shared" si="7"/>
-        <v>0.94400000000000261</v>
-      </c>
-    </row>
-    <row r="28" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B28" s="3">
-        <v>30</v>
-      </c>
-      <c r="C28" s="3">
-        <v>3.2389999999999999</v>
-      </c>
-      <c r="D28" s="7">
-        <v>2.4946000000000002</v>
-      </c>
-      <c r="E28" s="7">
-        <f t="shared" si="1"/>
-        <v>0.74439999999999973</v>
-      </c>
-      <c r="F28" s="7">
-        <f t="shared" si="2"/>
-        <v>1.4887999999999995</v>
-      </c>
-      <c r="G28" s="3">
-        <v>1.5</v>
-      </c>
-      <c r="H28" s="3">
-        <v>1.4883</v>
-      </c>
-      <c r="I28" s="7">
-        <f t="shared" si="6"/>
-        <v>1.1700000000000044E-2</v>
-      </c>
-      <c r="J28" s="3">
-        <f t="shared" si="7"/>
-        <v>0.78000000000000291</v>
-      </c>
-    </row>
-    <row r="29" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B29" s="3">
+        <v>4.1866666666666639</v>
+      </c>
+      <c r="K9" s="19">
+        <v>2.0230000000000001</v>
+      </c>
+    </row>
+    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B10" s="19">
         <v>35</v>
       </c>
-      <c r="C29" s="3">
+      <c r="C10" s="19">
         <v>3.3639999999999999</v>
       </c>
-      <c r="D29" s="7">
+      <c r="D10" s="20">
         <v>2.4946999999999999</v>
       </c>
-      <c r="E29" s="7">
+      <c r="E10" s="20">
         <f t="shared" si="1"/>
         <v>0.86929999999999996</v>
       </c>
-      <c r="F29" s="7">
-        <f t="shared" si="2"/>
+      <c r="F10" s="20">
+        <f t="shared" ref="F10:F13" si="4">2*E10</f>
         <v>1.7385999999999999</v>
       </c>
-      <c r="G29" s="3">
+      <c r="G10" s="19">
         <v>1.75</v>
       </c>
-      <c r="H29" s="3">
-        <v>1.7378</v>
-      </c>
-      <c r="I29" s="7">
-        <f t="shared" si="6"/>
-        <v>1.2199999999999989E-2</v>
-      </c>
-      <c r="J29" s="3">
-        <f t="shared" si="7"/>
-        <v>0.69714285714285651</v>
-      </c>
-    </row>
-    <row r="30" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B30" s="3">
+      <c r="H10" s="19">
+        <v>1.673</v>
+      </c>
+      <c r="I10" s="20">
+        <f t="shared" si="3"/>
+        <v>7.6999999999999957E-2</v>
+      </c>
+      <c r="J10" s="19">
+        <f t="shared" si="0"/>
+        <v>4.3999999999999977</v>
+      </c>
+      <c r="K10" s="19">
+        <v>2.0270000000000001</v>
+      </c>
+    </row>
+    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B11" s="19">
         <v>40</v>
       </c>
-      <c r="C30" s="3">
+      <c r="C11" s="19">
         <v>3.4891999999999999</v>
       </c>
-      <c r="D30" s="7">
+      <c r="D11" s="20">
         <v>2.4948999999999999</v>
       </c>
-      <c r="E30" s="7">
+      <c r="E11" s="20">
         <f t="shared" si="1"/>
         <v>0.99429999999999996</v>
       </c>
-      <c r="F30" s="7">
-        <f t="shared" si="2"/>
+      <c r="F11" s="20">
+        <f t="shared" si="4"/>
         <v>1.9885999999999999</v>
       </c>
-      <c r="G30" s="3">
+      <c r="G11" s="19">
         <v>2</v>
       </c>
-      <c r="H30" s="3">
-        <v>1.9884999999999999</v>
-      </c>
-      <c r="I30" s="7">
-        <f t="shared" si="6"/>
-        <v>1.1500000000000066E-2</v>
-      </c>
-      <c r="J30" s="3">
-        <f t="shared" si="7"/>
-        <v>0.57500000000000329</v>
-      </c>
-    </row>
-    <row r="31" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B31" s="3">
+      <c r="H11" s="19">
+        <v>1.9135</v>
+      </c>
+      <c r="I11" s="20">
+        <f t="shared" si="3"/>
+        <v>8.6500000000000021E-2</v>
+      </c>
+      <c r="J11" s="19">
+        <f t="shared" si="0"/>
+        <v>4.3250000000000011</v>
+      </c>
+      <c r="K11" s="19"/>
+    </row>
+    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B12" s="19">
         <v>45</v>
       </c>
-      <c r="C31" s="3">
+      <c r="C12" s="19">
         <v>3.6145</v>
       </c>
-      <c r="D31" s="7">
+      <c r="D12" s="20">
         <v>2.4950000000000001</v>
       </c>
-      <c r="E31" s="7">
+      <c r="E12" s="20">
         <f t="shared" si="1"/>
         <v>1.1194999999999999</v>
       </c>
-      <c r="F31" s="7">
-        <f t="shared" si="2"/>
+      <c r="F12" s="20">
+        <f t="shared" si="4"/>
         <v>2.2389999999999999</v>
       </c>
-      <c r="G31" s="3">
+      <c r="G12" s="19">
         <v>2.25</v>
       </c>
-      <c r="H31" s="3">
-        <v>2.2385000000000002</v>
-      </c>
-      <c r="I31" s="7">
-        <f t="shared" si="6"/>
-        <v>1.1499999999999844E-2</v>
-      </c>
-      <c r="J31" s="3">
-        <f t="shared" si="7"/>
-        <v>0.51111111111110419</v>
-      </c>
-    </row>
-    <row r="32" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B32" s="3">
+      <c r="H12" s="19">
+        <v>2.1539999999999999</v>
+      </c>
+      <c r="I12" s="20">
+        <f t="shared" si="3"/>
+        <v>9.6000000000000085E-2</v>
+      </c>
+      <c r="J12" s="19">
+        <f t="shared" si="0"/>
+        <v>4.266666666666671</v>
+      </c>
+      <c r="K12" s="19"/>
+    </row>
+    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B13" s="19">
         <v>50</v>
       </c>
-      <c r="C32" s="3">
+      <c r="C13" s="19">
         <v>3.7397</v>
       </c>
-      <c r="D32" s="7">
+      <c r="D13" s="20">
         <v>2.4952000000000001</v>
       </c>
-      <c r="E32" s="7">
+      <c r="E13" s="20">
         <f t="shared" si="1"/>
         <v>1.2444999999999999</v>
       </c>
-      <c r="F32" s="7">
-        <f t="shared" si="2"/>
+      <c r="F13" s="20">
+        <f t="shared" si="4"/>
         <v>2.4889999999999999</v>
       </c>
-      <c r="G32" s="3">
+      <c r="G13" s="19">
         <v>2.5</v>
       </c>
-      <c r="H32" s="3">
-        <v>2.4731999999999998</v>
-      </c>
-      <c r="I32" s="7">
-        <f t="shared" si="6"/>
-        <v>2.6800000000000157E-2</v>
-      </c>
-      <c r="J32" s="3">
-        <f t="shared" si="7"/>
-        <v>1.0720000000000063</v>
-      </c>
+      <c r="H13" s="19">
+        <v>2.395</v>
+      </c>
+      <c r="I13" s="20">
+        <f t="shared" si="3"/>
+        <v>0.10499999999999998</v>
+      </c>
+      <c r="J13" s="19">
+        <f t="shared" si="0"/>
+        <v>4.1999999999999993</v>
+      </c>
+      <c r="K13" s="19">
+        <v>2.0339999999999998</v>
+      </c>
+    </row>
+    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="K14" s="1"/>
+    </row>
+    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="K15" s="1"/>
+    </row>
+    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="K16" s="1"/>
+    </row>
+    <row r="17" spans="11:11" x14ac:dyDescent="0.35">
+      <c r="K17" s="1"/>
+    </row>
+    <row r="18" spans="11:11" x14ac:dyDescent="0.35">
+      <c r="K18" s="1"/>
+    </row>
+    <row r="19" spans="11:11" x14ac:dyDescent="0.35">
+      <c r="K19" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D00F4CA9-EF39-4B22-821D-9A3A0F70419D}">
+  <dimension ref="A3:H38"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="13.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.7265625" customWidth="1"/>
+    <col min="4" max="4" width="11.81640625" customWidth="1"/>
+    <col min="5" max="5" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.90625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.6328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="1:8" ht="26" x14ac:dyDescent="0.6">
+      <c r="A3" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" s="1"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D4" s="1"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D5" s="1"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D6" s="1"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="C7" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="D7" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="E7" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="F7" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="G7" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="H7" s="17" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B8" s="13"/>
+      <c r="C8" s="19">
+        <v>-50</v>
+      </c>
+      <c r="D8" s="19">
+        <v>-2.5</v>
+      </c>
+      <c r="E8" s="20">
+        <v>-2.5001000000000002</v>
+      </c>
+      <c r="F8" s="20">
+        <f>D8-E8</f>
+        <v>1.0000000000021103E-4</v>
+      </c>
+      <c r="G8" s="19">
+        <f t="shared" ref="G8:G34" si="0">(F8/D8)*100</f>
+        <v>-4.0000000000084412E-3</v>
+      </c>
+      <c r="H8" s="19">
+        <v>2.4620000000000002</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B9" s="13"/>
+      <c r="C9" s="19">
+        <v>-45</v>
+      </c>
+      <c r="D9" s="19">
+        <v>-2.25</v>
+      </c>
+      <c r="E9" s="20">
+        <v>-2.2492999999999999</v>
+      </c>
+      <c r="F9" s="20">
+        <f t="shared" ref="F9:F34" si="1">D9-E9</f>
+        <v>-7.0000000000014495E-4</v>
+      </c>
+      <c r="G9" s="19">
+        <f t="shared" si="0"/>
+        <v>3.1111111111117553E-2</v>
+      </c>
+      <c r="H9" s="19"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B10" s="13"/>
+      <c r="C10" s="19">
+        <v>-40</v>
+      </c>
+      <c r="D10" s="19">
+        <v>-2</v>
+      </c>
+      <c r="E10" s="20">
+        <v>-1.9987999999999999</v>
+      </c>
+      <c r="F10" s="20">
+        <f t="shared" si="1"/>
+        <v>-1.2000000000000899E-3</v>
+      </c>
+      <c r="G10" s="19">
+        <f t="shared" si="0"/>
+        <v>6.0000000000004494E-2</v>
+      </c>
+      <c r="H10" s="19">
+        <v>2.4624000000000001</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B11" s="13"/>
+      <c r="C11" s="19">
+        <v>-35</v>
+      </c>
+      <c r="D11" s="19">
+        <v>-1.75</v>
+      </c>
+      <c r="E11" s="20">
+        <v>-1.7477</v>
+      </c>
+      <c r="F11" s="20">
+        <f t="shared" si="1"/>
+        <v>-2.2999999999999687E-3</v>
+      </c>
+      <c r="G11" s="19">
+        <f t="shared" si="0"/>
+        <v>0.13142857142856965</v>
+      </c>
+      <c r="H11" s="19">
+        <v>2.4628000000000001</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="C12" s="19">
+        <v>-30</v>
+      </c>
+      <c r="D12" s="19">
+        <v>-1.5</v>
+      </c>
+      <c r="E12" s="20">
+        <v>-1.4964</v>
+      </c>
+      <c r="F12" s="20">
+        <f t="shared" si="1"/>
+        <v>-3.6000000000000476E-3</v>
+      </c>
+      <c r="G12" s="19">
+        <f t="shared" si="0"/>
+        <v>0.24000000000000318</v>
+      </c>
+      <c r="H12" s="19"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="C13" s="19">
+        <v>-25</v>
+      </c>
+      <c r="D13" s="19">
+        <v>-1.25</v>
+      </c>
+      <c r="E13" s="20">
+        <v>-1.2450000000000001</v>
+      </c>
+      <c r="F13" s="20">
+        <f t="shared" si="1"/>
+        <v>-4.9999999999998934E-3</v>
+      </c>
+      <c r="G13" s="19">
+        <f t="shared" si="0"/>
+        <v>0.39999999999999153</v>
+      </c>
+      <c r="H13" s="19">
+        <v>2.4628000000000001</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="C14" s="19">
+        <v>-20</v>
+      </c>
+      <c r="D14" s="19">
+        <v>-1</v>
+      </c>
+      <c r="E14" s="20">
+        <v>-0.99509999999999998</v>
+      </c>
+      <c r="F14" s="20">
+        <f t="shared" si="1"/>
+        <v>-4.9000000000000155E-3</v>
+      </c>
+      <c r="G14" s="19">
+        <f t="shared" si="0"/>
+        <v>0.49000000000000155</v>
+      </c>
+      <c r="H14" s="19"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="C15" s="19">
+        <v>-15</v>
+      </c>
+      <c r="D15" s="19">
+        <v>-0.75</v>
+      </c>
+      <c r="E15" s="20">
+        <v>-0.74650000000000005</v>
+      </c>
+      <c r="F15" s="20">
+        <f t="shared" si="1"/>
+        <v>-3.4999999999999476E-3</v>
+      </c>
+      <c r="G15" s="19">
+        <f t="shared" si="0"/>
+        <v>0.46666666666665968</v>
+      </c>
+      <c r="H15" s="19">
+        <v>2.4634999999999998</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="C16" s="19">
+        <v>-10</v>
+      </c>
+      <c r="D16" s="19">
+        <v>-0.5</v>
+      </c>
+      <c r="E16" s="20">
+        <v>-0.49349999999999999</v>
+      </c>
+      <c r="F16" s="20">
+        <f t="shared" si="1"/>
+        <v>-6.5000000000000058E-3</v>
+      </c>
+      <c r="G16" s="19">
+        <f t="shared" si="0"/>
+        <v>1.3000000000000012</v>
+      </c>
+      <c r="H16" s="19"/>
+    </row>
+    <row r="17" spans="3:8" x14ac:dyDescent="0.35">
+      <c r="C17" s="19">
+        <v>-8</v>
+      </c>
+      <c r="D17" s="19">
+        <v>-0.4</v>
+      </c>
+      <c r="E17" s="20">
+        <v>-0.3952</v>
+      </c>
+      <c r="F17" s="20">
+        <f t="shared" si="1"/>
+        <v>-4.8000000000000265E-3</v>
+      </c>
+      <c r="G17" s="19">
+        <f t="shared" si="0"/>
+        <v>1.2000000000000066</v>
+      </c>
+      <c r="H17" s="19"/>
+    </row>
+    <row r="18" spans="3:8" x14ac:dyDescent="0.35">
+      <c r="C18" s="19">
+        <v>-6</v>
+      </c>
+      <c r="D18" s="19">
+        <v>-0.3</v>
+      </c>
+      <c r="E18" s="20">
+        <v>-0.29299999999999998</v>
+      </c>
+      <c r="F18" s="20">
+        <f t="shared" si="1"/>
+        <v>-7.0000000000000062E-3</v>
+      </c>
+      <c r="G18" s="19">
+        <f t="shared" si="0"/>
+        <v>2.3333333333333357</v>
+      </c>
+      <c r="H18" s="19"/>
+    </row>
+    <row r="19" spans="3:8" x14ac:dyDescent="0.35">
+      <c r="C19" s="19">
+        <v>-4</v>
+      </c>
+      <c r="D19" s="19">
+        <v>-0.2</v>
+      </c>
+      <c r="E19" s="20">
+        <v>-0.19500000000000001</v>
+      </c>
+      <c r="F19" s="20">
+        <f t="shared" si="1"/>
+        <v>-5.0000000000000044E-3</v>
+      </c>
+      <c r="G19" s="19">
+        <f t="shared" si="0"/>
+        <v>2.5000000000000022</v>
+      </c>
+      <c r="H19" s="19"/>
+    </row>
+    <row r="20" spans="3:8" x14ac:dyDescent="0.35">
+      <c r="C20" s="19">
+        <v>-2</v>
+      </c>
+      <c r="D20" s="19">
+        <v>-0.1</v>
+      </c>
+      <c r="E20" s="20">
+        <v>-9.5799999999999996E-2</v>
+      </c>
+      <c r="F20" s="20">
+        <f t="shared" si="1"/>
+        <v>-4.2000000000000093E-3</v>
+      </c>
+      <c r="G20" s="19">
+        <f t="shared" si="0"/>
+        <v>4.2000000000000091</v>
+      </c>
+      <c r="H20" s="19"/>
+    </row>
+    <row r="21" spans="3:8" x14ac:dyDescent="0.35">
+      <c r="C21" s="19">
+        <v>0</v>
+      </c>
+      <c r="D21" s="19">
+        <v>0</v>
+      </c>
+      <c r="E21" s="20">
+        <v>1E-4</v>
+      </c>
+      <c r="F21" s="20">
+        <f t="shared" si="1"/>
+        <v>-1E-4</v>
+      </c>
+      <c r="G21" s="19" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H21" s="19">
+        <v>2.4660000000000002</v>
+      </c>
+    </row>
+    <row r="22" spans="3:8" x14ac:dyDescent="0.35">
+      <c r="C22" s="19">
+        <v>2</v>
+      </c>
+      <c r="D22" s="19">
+        <v>0.1</v>
+      </c>
+      <c r="E22" s="20">
+        <v>9.5200000000000007E-2</v>
+      </c>
+      <c r="F22" s="20">
+        <f t="shared" si="1"/>
+        <v>4.7999999999999987E-3</v>
+      </c>
+      <c r="G22" s="19">
+        <f t="shared" si="0"/>
+        <v>4.7999999999999989</v>
+      </c>
+      <c r="H22" s="19"/>
+    </row>
+    <row r="23" spans="3:8" x14ac:dyDescent="0.35">
+      <c r="C23" s="19">
+        <v>4</v>
+      </c>
+      <c r="D23" s="19">
+        <v>0.2</v>
+      </c>
+      <c r="E23" s="20">
+        <v>0.192</v>
+      </c>
+      <c r="F23" s="20">
+        <f t="shared" si="1"/>
+        <v>8.0000000000000071E-3</v>
+      </c>
+      <c r="G23" s="19">
+        <f t="shared" si="0"/>
+        <v>4.0000000000000036</v>
+      </c>
+      <c r="H23" s="19"/>
+    </row>
+    <row r="24" spans="3:8" x14ac:dyDescent="0.35">
+      <c r="C24" s="19">
+        <v>6</v>
+      </c>
+      <c r="D24" s="19">
+        <v>0.3</v>
+      </c>
+      <c r="E24" s="20">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="F24" s="20">
+        <f t="shared" si="1"/>
+        <v>1.0000000000000009E-2</v>
+      </c>
+      <c r="G24" s="19">
+        <f t="shared" si="0"/>
+        <v>3.3333333333333366</v>
+      </c>
+      <c r="H24" s="19"/>
+    </row>
+    <row r="25" spans="3:8" x14ac:dyDescent="0.35">
+      <c r="C25" s="19">
+        <v>8</v>
+      </c>
+      <c r="D25" s="19">
+        <v>0.4</v>
+      </c>
+      <c r="E25" s="20">
+        <v>0.39200000000000002</v>
+      </c>
+      <c r="F25" s="20">
+        <f t="shared" si="1"/>
+        <v>8.0000000000000071E-3</v>
+      </c>
+      <c r="G25" s="19">
+        <f t="shared" si="0"/>
+        <v>2.0000000000000018</v>
+      </c>
+      <c r="H25" s="19"/>
+    </row>
+    <row r="26" spans="3:8" x14ac:dyDescent="0.35">
+      <c r="C26" s="19">
+        <v>10</v>
+      </c>
+      <c r="D26" s="19">
+        <v>0.5</v>
+      </c>
+      <c r="E26" s="20">
+        <v>0.4929</v>
+      </c>
+      <c r="F26" s="20">
+        <f t="shared" si="1"/>
+        <v>7.0999999999999952E-3</v>
+      </c>
+      <c r="G26" s="19">
+        <f t="shared" si="0"/>
+        <v>1.419999999999999</v>
+      </c>
+      <c r="H26" s="19"/>
+    </row>
+    <row r="27" spans="3:8" x14ac:dyDescent="0.35">
+      <c r="C27" s="19">
+        <v>15</v>
+      </c>
+      <c r="D27" s="19">
+        <v>0.75</v>
+      </c>
+      <c r="E27" s="19">
+        <v>0.74560000000000004</v>
+      </c>
+      <c r="F27" s="20">
+        <f t="shared" si="1"/>
+        <v>4.3999999999999595E-3</v>
+      </c>
+      <c r="G27" s="19">
+        <f t="shared" si="0"/>
+        <v>0.58666666666666134</v>
+      </c>
+      <c r="H27" s="21"/>
+    </row>
+    <row r="28" spans="3:8" x14ac:dyDescent="0.35">
+      <c r="C28" s="19">
+        <v>20</v>
+      </c>
+      <c r="D28" s="19">
+        <v>1</v>
+      </c>
+      <c r="E28" s="19">
+        <v>0.99399999999999999</v>
+      </c>
+      <c r="F28" s="20">
+        <f t="shared" si="1"/>
+        <v>6.0000000000000053E-3</v>
+      </c>
+      <c r="G28" s="19">
+        <f t="shared" si="0"/>
+        <v>0.60000000000000053</v>
+      </c>
+      <c r="H28" s="19">
+        <v>2.4634999999999998</v>
+      </c>
+    </row>
+    <row r="29" spans="3:8" x14ac:dyDescent="0.35">
+      <c r="C29" s="19">
+        <v>25</v>
+      </c>
+      <c r="D29" s="19">
+        <v>1.25</v>
+      </c>
+      <c r="E29" s="19">
+        <v>1.244</v>
+      </c>
+      <c r="F29" s="20">
+        <f t="shared" si="1"/>
+        <v>6.0000000000000053E-3</v>
+      </c>
+      <c r="G29" s="19">
+        <f t="shared" si="0"/>
+        <v>0.48000000000000037</v>
+      </c>
+      <c r="H29" s="19"/>
+    </row>
+    <row r="30" spans="3:8" x14ac:dyDescent="0.35">
+      <c r="C30" s="19">
+        <v>30</v>
+      </c>
+      <c r="D30" s="19">
+        <v>1.5</v>
+      </c>
+      <c r="E30" s="19">
+        <v>1.4955000000000001</v>
+      </c>
+      <c r="F30" s="20">
+        <f t="shared" si="1"/>
+        <v>4.4999999999999485E-3</v>
+      </c>
+      <c r="G30" s="19">
+        <f t="shared" si="0"/>
+        <v>0.2999999999999966</v>
+      </c>
+      <c r="H30" s="19">
+        <v>2.4630000000000001</v>
+      </c>
+    </row>
+    <row r="31" spans="3:8" x14ac:dyDescent="0.35">
+      <c r="C31" s="19">
+        <v>35</v>
+      </c>
+      <c r="D31" s="19">
+        <v>1.75</v>
+      </c>
+      <c r="E31" s="19">
+        <v>1.7455000000000001</v>
+      </c>
+      <c r="F31" s="20">
+        <f t="shared" si="1"/>
+        <v>4.4999999999999485E-3</v>
+      </c>
+      <c r="G31" s="19">
+        <f t="shared" si="0"/>
+        <v>0.25714285714285418</v>
+      </c>
+      <c r="H31" s="19"/>
+    </row>
+    <row r="32" spans="3:8" x14ac:dyDescent="0.35">
+      <c r="C32" s="19">
+        <v>40</v>
+      </c>
+      <c r="D32" s="19">
+        <v>2</v>
+      </c>
+      <c r="E32" s="19">
+        <v>1.9963</v>
+      </c>
+      <c r="F32" s="20">
+        <f t="shared" si="1"/>
+        <v>3.7000000000000366E-3</v>
+      </c>
+      <c r="G32" s="19">
+        <f t="shared" si="0"/>
+        <v>0.18500000000000183</v>
+      </c>
+      <c r="H32" s="19">
+        <v>2.4624999999999999</v>
+      </c>
+    </row>
+    <row r="33" spans="3:8" x14ac:dyDescent="0.35">
+      <c r="C33" s="19">
+        <v>45</v>
+      </c>
+      <c r="D33" s="19">
+        <v>2.25</v>
+      </c>
+      <c r="E33" s="19">
+        <v>2.2464</v>
+      </c>
+      <c r="F33" s="20">
+        <f t="shared" si="1"/>
+        <v>3.6000000000000476E-3</v>
+      </c>
+      <c r="G33" s="19">
+        <f t="shared" si="0"/>
+        <v>0.16000000000000211</v>
+      </c>
+      <c r="H33" s="19"/>
+    </row>
+    <row r="34" spans="3:8" x14ac:dyDescent="0.35">
+      <c r="C34" s="19">
+        <v>50</v>
+      </c>
+      <c r="D34" s="19">
+        <v>2.5</v>
+      </c>
+      <c r="E34" s="19">
+        <v>2.4967000000000001</v>
+      </c>
+      <c r="F34" s="20">
+        <f t="shared" si="1"/>
+        <v>3.2999999999998586E-3</v>
+      </c>
+      <c r="G34" s="19">
+        <f t="shared" si="0"/>
+        <v>0.13199999999999434</v>
+      </c>
+      <c r="H34" s="19">
+        <v>2.4620000000000002</v>
+      </c>
+    </row>
+    <row r="35" spans="3:8" x14ac:dyDescent="0.35">
+      <c r="D35" s="1"/>
+    </row>
+    <row r="36" spans="3:8" x14ac:dyDescent="0.35">
+      <c r="D36" s="1"/>
+    </row>
+    <row r="37" spans="3:8" x14ac:dyDescent="0.35">
+      <c r="D37" s="1"/>
+    </row>
+    <row r="38" spans="3:8" x14ac:dyDescent="0.35">
+      <c r="D38" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>